<commit_message>
Related-record stories: guard resource/time maps from creating tasks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Ctr8mgkRhw8W6DYxzjejb
</commit_message>
<xml_diff>
--- a/docs/rm_story_related_records.xlsx
+++ b/docs/rm_story_related_records.xlsx
@@ -818,7 +818,7 @@
 - Adaptive: Data Source 'Adaptive Resources - API' (STRY0067506) loads one row per resource link with Project Correlation ID = the work item (task or project) and Resource Email.
 - Transform map u_import_adaptive_resources -&gt; pm_project_task, coalesce on correlation_id = the task's correlation id (field map [Script] -&gt; correlation_id returning source.u_project_correlation_id).
 - onBefore: first resource on a task -&gt; assigned_to; further resources are added to additional_assignee_list (no duplicates). Users matched on email; no match -&gt; logged, left blank.
-- Links whose work item is a project (ADAPTIVE:/Project/...) update additional_assignee_list on pm_project.
+- onBefore also: if no pm_project_task has that correlation_id, ignore = true (this map must never create tasks). Links whose work item is a project (ADAPTIVE:/Project/...) are skipped here; a second map on the same staging table -&gt; pm_project (same rules) adds them to the project's additional_assignee_list.
 - Asana: no separate feed - assignee and followers already come with the Work Plan (NEW-11/NEW-12).
 - Done when the pilot tasks show the same people as Adaptive.</t>
         </is>
@@ -827,7 +827,7 @@
         <is>
           <t>&lt;p&gt;Built on what is proven in Dev: system properties x_mig.adaptive.url / x_mig.adaptive.key / x_mig.asana.token / x_mig.asana.project_gid, and the &amp;#x27;Adaptive Projects - API&amp;#x27; Data Source (PRJ0010675 loaded from the API). Keys: correlation_id = &amp;quot;ADAPTIVE:&amp;quot; + Adaptive id (e.g. ADAPTIVE:/Project/5afh...) or &amp;quot;ASANA:&amp;quot; + Asana gid. Scripts are in the repo folder servicenow/.&lt;/p&gt;
 &lt;p&gt;Scope: put the people on the tasks (assigned_to + additional_assignee_list). Full Resource Management (resource plans / allocations) is NOT in this story (decision D2). Rate models are removed unless time is loaded as time cards (decision D3).&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;Adaptive: Data Source &amp;#x27;Adaptive Resources - API&amp;#x27; (STRY0067506) loads one row per resource link with Project Correlation ID = the work item (task or project) and Resource Email.&lt;/li&gt;&lt;li&gt;Transform map u_import_adaptive_resources -&amp;gt; pm_project_task, coalesce on correlation_id = the task&amp;#x27;s correlation id (field map [Script] -&amp;gt; correlation_id returning source.u_project_correlation_id).&lt;/li&gt;&lt;li&gt;onBefore: first resource on a task -&amp;gt; assigned_to; further resources are added to additional_assignee_list (no duplicates). Users matched on email; no match -&amp;gt; logged, left blank.&lt;/li&gt;&lt;li&gt;Links whose work item is a project (ADAPTIVE:/Project/...) update additional_assignee_list on pm_project.&lt;/li&gt;&lt;li&gt;Asana: no separate feed - assignee and followers already come with the Work Plan (NEW-11/NEW-12).&lt;/li&gt;&lt;li&gt;Done when the pilot tasks show the same people as Adaptive.&lt;/li&gt;&lt;/ul&gt;</t>
+&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;Adaptive: Data Source &amp;#x27;Adaptive Resources - API&amp;#x27; (STRY0067506) loads one row per resource link with Project Correlation ID = the work item (task or project) and Resource Email.&lt;/li&gt;&lt;li&gt;Transform map u_import_adaptive_resources -&amp;gt; pm_project_task, coalesce on correlation_id = the task&amp;#x27;s correlation id (field map [Script] -&amp;gt; correlation_id returning source.u_project_correlation_id).&lt;/li&gt;&lt;li&gt;onBefore: first resource on a task -&amp;gt; assigned_to; further resources are added to additional_assignee_list (no duplicates). Users matched on email; no match -&amp;gt; logged, left blank.&lt;/li&gt;&lt;li&gt;onBefore also: if no pm_project_task has that correlation_id, ignore = true (this map must never create tasks). Links whose work item is a project (ADAPTIVE:/Project/...) are skipped here; a second map on the same staging table -&amp;gt; pm_project (same rules) adds them to the project&amp;#x27;s additional_assignee_list.&lt;/li&gt;&lt;li&gt;Asana: no separate feed - assignee and followers already come with the Work Plan (NEW-11/NEW-12).&lt;/li&gt;&lt;li&gt;Done when the pilot tasks show the same people as Adaptive.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
 Decision D3. Option A (this story): carry total hours already worked onto each task, so actuals are not lost. Option B (time cards per user per week, with rate models) adds cost records, approvals and fiscal periods; only if the client needs timesheet history in ServiceNow.
 - Adaptive: Data Source 'Adaptive Time - API' (STRY0067506) on entity [CONFIRM] (e.g. Timesheet), fields [CONFIRM] (reported by, work item, date, duration).
 - Its script sums hours per work item before inserting: one staging row per task with Project Correlation ID (= the task) and Total Hours.
-- Transform -&gt; pm_project_task, coalesce via [Script] -&gt; correlation_id = source.u_project_correlation_id; Total Hours -&gt; the task's Actual effort field (dev confirms the field name in the pm_project_task dictionary).
+- Transform -&gt; pm_project_task, coalesce via [Script] -&gt; correlation_id = source.u_project_correlation_id; Total Hours -&gt; the task's Actual effort field (dev confirms the field name in the pm_project_task dictionary). onBefore: if no pm_project_task has that correlation_id, ignore = true (never create tasks from this map).
 - Asana: only if Discovery shows actual_time_minutes; then the Work Plan script also fills Total Hours (minutes / 60).
 - Done when pilot task actual effort equals the Adaptive totals (spot-check 5 tasks).</t>
         </is>
@@ -865,7 +865,7 @@
         <is>
           <t>&lt;p&gt;Built on what is proven in Dev: system properties x_mig.adaptive.url / x_mig.adaptive.key / x_mig.asana.token / x_mig.asana.project_gid, and the &amp;#x27;Adaptive Projects - API&amp;#x27; Data Source (PRJ0010675 loaded from the API). Keys: correlation_id = &amp;quot;ADAPTIVE:&amp;quot; + Adaptive id (e.g. ADAPTIVE:/Project/5afh...) or &amp;quot;ASANA:&amp;quot; + Asana gid. Scripts are in the repo folder servicenow/.&lt;/p&gt;
 &lt;p&gt;Decision D3. Option A (this story): carry total hours already worked onto each task, so actuals are not lost. Option B (time cards per user per week, with rate models) adds cost records, approvals and fiscal periods; only if the client needs timesheet history in ServiceNow.&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;Adaptive: Data Source &amp;#x27;Adaptive Time - API&amp;#x27; (STRY0067506) on entity [CONFIRM] (e.g. Timesheet), fields [CONFIRM] (reported by, work item, date, duration).&lt;/li&gt;&lt;li&gt;Its script sums hours per work item before inserting: one staging row per task with Project Correlation ID (= the task) and Total Hours.&lt;/li&gt;&lt;li&gt;Transform -&amp;gt; pm_project_task, coalesce via [Script] -&amp;gt; correlation_id = source.u_project_correlation_id; Total Hours -&amp;gt; the task&amp;#x27;s Actual effort field (dev confirms the field name in the pm_project_task dictionary).&lt;/li&gt;&lt;li&gt;Asana: only if Discovery shows actual_time_minutes; then the Work Plan script also fills Total Hours (minutes / 60).&lt;/li&gt;&lt;li&gt;Done when pilot task actual effort equals the Adaptive totals (spot-check 5 tasks).&lt;/li&gt;&lt;/ul&gt;</t>
+&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;Adaptive: Data Source &amp;#x27;Adaptive Time - API&amp;#x27; (STRY0067506) on entity [CONFIRM] (e.g. Timesheet), fields [CONFIRM] (reported by, work item, date, duration).&lt;/li&gt;&lt;li&gt;Its script sums hours per work item before inserting: one staging row per task with Project Correlation ID (= the task) and Total Hours.&lt;/li&gt;&lt;li&gt;Transform -&amp;gt; pm_project_task, coalesce via [Script] -&amp;gt; correlation_id = source.u_project_correlation_id; Total Hours -&amp;gt; the task&amp;#x27;s Actual effort field (dev confirms the field name in the pm_project_task dictionary). onBefore: if no pm_project_task has that correlation_id, ignore = true (never create tasks from this map).&lt;/li&gt;&lt;li&gt;Asana: only if Discovery shows actual_time_minutes; then the Work Plan script also fills Total Hours (minutes / 60).&lt;/li&gt;&lt;li&gt;Done when pilot task actual effort equals the Adaptive totals (spot-check 5 tasks).&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>